<commit_message>
prepare ballot (#150) 60ff5e724cd975291679069f54153992c720acc8
</commit_message>
<xml_diff>
--- a/ig/main/CodeSystem-as-cs-intern-id-systems.xlsx
+++ b/ig/main/CodeSystem-as-cs-intern-id-systems.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0-ballot-2</t>
+    <t>1.0.0-ballot-3</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-12-19T08:36:38+00:00</t>
+    <t>2023-12-19T15:11:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>